<commit_message>
Aponta o ciclo de 10 min para o CSV organizado e republica as pendencias no Pages.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/PENDENCIAS_SINCRONISMO.xlsx
+++ b/PENDENCIAS_SINCRONISMO.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>25/08/2026 18:52</t>
+          <t>25/08/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>25/08/2026 18:52</t>
+          <t>25/08/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -45172,7 +45172,7 @@
       </c>
       <c r="K533" t="inlineStr">
         <is>
-          <t>VTC - YASMIN SILVA TEIXEIRA</t>
+          <t>VTC - ANDERSON DE SOUZA SONCINE</t>
         </is>
       </c>
       <c r="L533" t="inlineStr">
@@ -45182,7 +45182,7 @@
       </c>
       <c r="M533" t="inlineStr">
         <is>
-          <t>25/08/26 16:47</t>
+          <t>25/08/26 18:59</t>
         </is>
       </c>
       <c r="N533" t="inlineStr">

</xml_diff>